<commit_message>
update all sofa titles - add USB Cup Holders for W1361 series
</commit_message>
<xml_diff>
--- a/KEIKI_SofaBed_新标题.xlsx
+++ b/KEIKI_SofaBed_新标题.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>KEIKI 83" 4Seat Modular Sectional Sleeper Pull Out Bed Corduroy Sofa Couch with Chaise Storage Reversible for Living Room Flexible Layout Comfy Lounge Black</t>
+          <t>KEIKI 83" 4Seat Modular Sectional Sleeper Pull Out Bed Corduroy Sofa Couch with Chaise Storage Reversible for Living Room Flexible Layout USB Cup Holders Comfy Lounge Black</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>KEIKI 83" 4Seat Modular Sectional Sleeper Pull Out Bed Corduroy Sofa Couch with Chaise Storage Reversible for Living Room Flexible Layout Comfy Lounge Grey</t>
+          <t>KEIKI 83" 4Seat Modular Sectional Sleeper Pull Out Bed Corduroy Sofa Couch with Chaise Storage Reversible for Living Room Flexible Layout USB Cup Holders Comfy Lounge Grey</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>KEIKI 83" 4Seat Modular Sectional Sleeper Pull Out Bed Corduroy Sofa Couch with Chaise Storage Reversible for Living Room Flexible Layout Comfy Lounge Orange</t>
+          <t>KEIKI 83" 4Seat Modular Sectional Sleeper Pull Out Bed Corduroy Sofa Couch with Chaise Storage Reversible for Living Room Flexible Layout USB Cup Holders Comfy Lounge Orange</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>KEIKI 83" 4Seat Modular Sectional Sleeper Pull Out Bed Corduroy Sofa Couch with Chaise Storage Reversible for Living Room Flexible Layout Comfy Lounge White</t>
+          <t>KEIKI 83" 4Seat Modular Sectional Sleeper Pull Out Bed Corduroy Sofa Couch with Chaise Storage Reversible for Living Room Flexible Layout USB Cup Holders Comfy Lounge White</t>
         </is>
       </c>
     </row>

</xml_diff>